<commit_message>
update(PushpendraSinghAITech): consolidated website directory (12 unique websites) - 2026-10-25 10:09:08
</commit_message>
<xml_diff>
--- a/📁 PushpendraSinghAITech/📊 PushpendraSinghAITech_Websites_Master_List.xlsx
+++ b/📁 PushpendraSinghAITech/📊 PushpendraSinghAITech_Websites_Master_List.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -521,7 +521,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>How to use muse ai in india</t>
+          <t>TinyWow</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -531,15 +531,15 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Online productivity utilities: how to use muse ai in India • Online productivity utilities: Jio IPO: Global Investors Se Lekar India ke Top MFs Tak • Online productivity utilities: How to Create Long AI Videos with Google Gemini • Online productivity utilities: Instagram's new comment image feature (Channel me kul 193 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: 200+ free online utility tools: PDF editing/converting/merging, image background removal, file compression, video tools, and AI writing. (Channel me kul 184 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>193 videos (Primary: https://www.youtube.com/shorts/u7WYpGiqnqU)</t>
+          <t>184 videos (Primary: https://www.youtube.com/shorts/u7WYpGiqnqU)</t>
         </is>
       </c>
     </row>
@@ -581,145 +581,295 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Tribit stormbox blast 2 200w p</t>
+          <t>Lovart AI</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>https://toools.design</t>
+          <t>https://lovart.ai</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Creative design utility: TRIBIT StormBox Blast 2 200W Party Speaker Review • Creative design utility: Top 3 Bawal Android Apps you must know • Creative design utility: How to Create viral torch videos of cartoon characters using Al • Creative design utility: Top 3 Useful android Apps (Channel me kul 36 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: AI-driven visual design tool and artistic creative generator for prompts and graphic media.</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>36 videos (Primary: https://www.youtube.com/shorts/8Fz0_CWJesk)</t>
+          <t>Create Viral Images Using Google Nano Banana (4VYDw6dRg7o)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>🎵 Audio, Voice &amp; Music</t>
+          <t>🎨 Design, 3D &amp; Graphics</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Your own songs like modi ai songs</t>
+          <t>Toools.design</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://vocalremover.org</t>
+          <t>https://toools.design</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye kar sakte hain: Audio manipulation: Create your own songs like Modi ai Songs</t>
+          <t>Is website se ye sab kar sakte hain: Curated repository of 1,000+ modern design tools, mockups, typography, illustration packs, and UI kits. (Channel me kul 38 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Create your own songs like Modi ai Songs (https://www.youtube.com/shorts/NmdPHJpldSo)</t>
+          <t>38 videos (Primary: https://www.youtube.com/shorts/8Fz0_CWJesk)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>💻 Coding &amp; Web Development</t>
+          <t>🎵 Audio, Voice &amp; Music</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Whatsapp &amp; telegram sim bindin</t>
+          <t>Udio</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://replit.com</t>
+          <t>https://udio.com</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Development &amp; code features: WhatsApp &amp; Telegram SIM Binding Rule 2026 • Development &amp; code features: WhatsApp 2 Features ! • Development &amp; code features: New E-rickshaw control app • Development &amp; code features: 3 Bawal Android Apps you must know (Channel me kul 53 alag-alag videos me featured)</t>
+          <t>Is website se ye kar sakte hain: High-fidelity AI music generation engine capable of generating full tracks from prompts.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>53 videos (Primary: D-nIf-3u4cY)</t>
+          <t>Top 5 best online tools for pdf, video editing, audio, image editing and much more (https://www.youtube.com/shorts/VgDZcJg9uBM)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>📚 Learning, Study &amp; Research</t>
+          <t>🎵 Audio, Voice &amp; Music</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>100+ free offers for students</t>
+          <t>Vocal Remover</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>https://quillbot.com</t>
+          <t>https://vocalremover.org</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Is website se ye sab kar sakte hain: Study &amp; academic utility: 100+ Free Offers for Students • Study &amp; academic utility: Explore Free Student Courses on the Best Government Website • Study &amp; academic utility: Best Website for Students • Study &amp; academic utility: Free coaching Classes for All Students (Channel me kul 9 alag-alag videos me featured)</t>
+          <t>Is website se ye sab kar sakte hain: AI-powered online audio tool that isolates vocals and instrumental tracks for free. (Channel me kul 2 alag-alag videos me featured)</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>9 videos (Primary: ooEpOTfcNNc)</t>
+          <t>2 videos (Primary: https://www.youtube.com/shorts/NczrBzD8qsU)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>💻 Coding &amp; Web Development</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Replit</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://replit.com</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Collaborative browser-based IDE, AI code generation, and instant cloud application deployment workspace. (Channel me kul 52 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>52 videos (Primary: D-nIf-3u4cY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>📚 Learning, Study &amp; Research</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>QuillBot</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>https://quillbot.com</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: AI paraphrasing, grammar checking, academic summarization, plagiarism detection, and student thesis writing assistance. (Channel me kul 8 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>8 videos (Primary: ooEpOTfcNNc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>🤖 AI &amp; Machine Learning Tools</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 best websites for all viral </t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://chatgpt.com</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Conversational AI assistant by OpenAI for answering questions, coding, research, writing, and problem solving. (Channel me kul 8 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>8 videos (Primary: https://www.youtube.com/shorts/U9zVSml2BKI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Google Gemini</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>https://gemini.google.com</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Multimodal conversational AI model by Google for advanced reasoning, coding, search, and Google Workspace integration. (Channel me kul 9 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>9 videos (Primary: yA9Tj0BpOVg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Perplexity AI</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://perplexity.ai</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Conversational AI search engine delivering verified answers with real-time web citations and academic research papers.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Get Perplexity Pro Worth 17,000 FREE with Airtel (Full Guide) (https://www.youtube.com/shorts/wYZ7nmda10M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>🤖 AI &amp; Machine Learning Tools</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Toolify.ai</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>https://toolify.ai</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Is website se ye sab kar sakte hain: AI features: 3 Best websites for all viral prompts for ChatGPT, Gemini, Claude and other AI • AI features: Google Gemini Prompt to Create Your Photo in IPL Team Jersey • AI features: 5 Hidden Websites With 500+ Online Tools • AI features: Best Google Gemini Prompt (Channel me kul 31 alag-alag videos me featured)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>31 videos (Primary: https://www.youtube.com/shorts/U9zVSml2BKI)</t>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Is website se ye sab kar sakte hain: Comprehensive global directory and discovery engine indexing 10,000+ AI software tools, models, and apps updated daily. (Channel me kul 19 alag-alag videos me featured)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>19 videos (Primary: https://www.youtube.com/shorts/IX-WqZ_L2Jo)</t>
         </is>
       </c>
     </row>
@@ -732,6 +882,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>